<commit_message>
Wire up Gemini API key; confirm connectivity end to end
- GEMINI_API_KEY set as a Railway environment variable (not committed,
  not printed anywhere in the repo)
- scripts/test_llm_connection.py: lists available models and does a
  real generateContent round-trip. First run caught that the obvious
  model name (gemini-2.5-flash) is already deprecated for new callers;
  switched to Google's own "gemini-flash-latest" alias instead, which
  stays current automatically rather than needing to be bumped by hand
- Capstone Team Plan.xlsx: decision #9 (LLM provider) marked resolved

Verified live: railway run python scripts/test_llm_connection.py
-> SUCCESS, model replied 'OK'

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Capstone Team Plan.xlsx
+++ b/Capstone Team Plan.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>OPEN — not yet chosen. Needed before AI agents can be wired to a real model.</t>
+          <t>RESOLVED — Google Gemini. Model: gemini-flash-latest (Google-maintained alias, avoids hardcoding a version that goes stale). Key is live in Railway (GEMINI_API_KEY). Connectivity smoke-tested successfully (scripts/test_llm_connection.py).</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>YES — must decide this week</t>
+          <t>No — done</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>This is Claude's first-cut assignment based on the only real signal available (Rahul = group admin, Sweta has driven direction) — not a claim about anyone's actual skills. Swap names in under 2 minutes on the call; the roles and responsibilities themselves are the part that's actually decided.</t>

</xml_diff>